<commit_message>
sociaal-wonen: bronbestanden en werkingsgebieden uit Toelichting-blad van de xlsx
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/sociaal-wonen/public/data/sociaal-wonen-alle-gegevens.xlsx
+++ b/apps/sociaal-wonen/public/data/sociaal-wonen-alle-gegevens.xlsx
@@ -26621,7 +26621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -26642,201 +26642,194 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Bronbestanden: 2026_08_14_KTP.xlsx, 2026_08_14_MJP.xlsx. Werkingsgebieden: Woonmaatschappijen in kaart (januari 2025).</t>
-        </is>
-      </c>
+      <c r="A3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr"/>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Planningen</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Planningen</t>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Korte termijn: Verrichtingen die klaar zijn voor aanbesteding.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Korte termijn: Verrichtingen die klaar zijn voor aanbesteding.</t>
+          <t>Lange termijn: Verrichtingen waarvoor een voorontwerp werd geadviseerd.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Lange termijn: Verrichtingen waarvoor een voorontwerp werd geadviseerd.</t>
+          <t>KT en LT zijn twee afzonderlijke planningen. Tel ze niet bij elkaar op.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>KT en LT zijn twee afzonderlijke planningen. Tel ze niet bij elkaar op.</t>
-        </is>
-      </c>
+      <c r="A8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Opbouw van het blad Gegevens</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Opbouw van het blad Gegevens</t>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Een rij per waarneming. Kolom Planning onderscheidt korte en lange termijn, kolom Niveau zegt waarvoor een rij staat.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Een rij per waarneming. Kolom Planning onderscheidt korte en lange termijn, kolom Niveau zegt waarvoor een rij staat.</t>
+          <t>Niveau Project (enkel korte termijn): een rij per verrichting, met projectomschrijving en datum opname programmatie.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Niveau Project (enkel korte termijn): een rij per verrichting, met projectomschrijving en datum opname programmatie.</t>
+          <t>Niveau Geaggregeerd (lange termijn): een rij per combinatie van woonmaatschappij, gemeente, soort werken, type en procedure. Projectdetails zijn voor de lange termijn niet beschikbaar.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Niveau Geaggregeerd (lange termijn): een rij per combinatie van woonmaatschappij, gemeente, soort werken, type en procedure. Projectdetails zijn voor de lange termijn niet beschikbaar.</t>
+          <t>Interne dossiernummers (Woonproject, Verrichting) staan niet in dit bestand. De SSI-bladen zijn niet inbegrepen, omdat ze overlappen met de gewone planning.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Interne dossiernummers (Woonproject, Verrichting) staan niet in dit bestand. De SSI-bladen zijn niet inbegrepen, omdat ze overlappen met de gewone planning.</t>
-        </is>
-      </c>
+      <c r="A14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr"/>
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Kolommen</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Kolommen</t>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Huurwoningen: Aantal huurwoningen dat zal gerealiseerd worden. Bij renovatie gaat het om bestaande woningen waarvan de ingreep beperkt kan zijn (bv. raamcontracten of beperkte renovatie). Vergelijk bedragen per woning daarom enkel binnen hetzelfde soort werken.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Huurwoningen: Aantal huurwoningen dat zal gerealiseerd worden. Bij renovatie gaat het om bestaande woningen waarvan de ingreep beperkt kan zijn (bv. raamcontracten of beperkte renovatie). Vergelijk bedragen per woning daarom enkel binnen hetzelfde soort werken.</t>
+          <t>Kostprijs (EUR): Geraamde kostprijs van de werken.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Kostprijs (EUR): Geraamde kostprijs van de werken.</t>
+          <t>Maximumprijs VMSW (EUR): FS4-plafond. Niet voor elke rij ingevuld.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Maximumprijs VMSW (EUR): FS4-plafond. Niet voor elke rij ingevuld.</t>
+          <t>Bedrag UP (EUR): Subsidiabel bedrag (berekend op basis van kostprijs en maximumprijs).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Bedrag UP (EUR): Subsidiabel bedrag (berekend op basis van kostprijs en maximumprijs).</t>
+          <t>Datum opname programmatie: Datum opname programmatie (kolom Datum Beslissing in de bron).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Datum opname programmatie: Datum opname programmatie (kolom Datum Beslissing in de bron).</t>
+          <t>Procedure: de kolom Extra info uit de bron, bv. CBO, Modulair Wonen, Design &amp; Build, raamcontract, beperkte renovatie. Leeg als niets vermeld is.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Procedure: de kolom Extra info uit de bron, bv. CBO, Modulair Wonen, Design &amp; Build, raamcontract, beperkte renovatie. Leeg als niets vermeld is.</t>
+          <t>Aantal verrichtingen: aantal verrichtingen achter de rij (1 bij niveau Project).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Aantal verrichtingen: aantal verrichtingen achter de rij (1 bij niveau Project).</t>
+          <t>Provincie en gemeente zijn afgeleid uit de NIS-code van de gemeente, niet uit de bronkolom. Rijen zonder eenduidige gemeente hebben geen NIS-code.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Provincie en gemeente zijn afgeleid uit de NIS-code van de gemeente, niet uit de bronkolom. Rijen zonder eenduidige gemeente hebben geen NIS-code.</t>
+          <t>Herhaalde huurwaarden binnen een verrichting zijn niet gecorrigeerd, zodat de totalen overeenkomen met de totaalrijen van VMSW.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Herhaalde huurwaarden binnen een verrichting zijn niet gecorrigeerd, zodat de totalen overeenkomen met de totaalrijen van VMSW.</t>
-        </is>
-      </c>
+      <c r="A25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Types verrichting</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Types verrichting</t>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>NB: Nieuwbouw</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>NB: Nieuwbouw</t>
+          <t>VVP: Vervangingsbouw verworven patrimonium</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>VVP: Vervangingsbouw verworven patrimonium</t>
+          <t>RVP: Renovatie verworven patrimonium</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>RVP: Renovatie verworven patrimonium</t>
+          <t>GW: Aankoop goede woning</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>GW: Aankoop goede woning</t>
+          <t>VEP: Vervangingsbouw eigen patrimonium</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>VEP: Vervangingsbouw eigen patrimonium</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>REP: Renovatie eigen patrimonium</t>
         </is>

</xml_diff>

<commit_message>
fix(sociaal-wonen): remove requested Excel explanation rows
Remove two notes from the download and its generator without changing the data.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/apps/sociaal-wonen/public/data/sociaal-wonen-alle-gegevens.xlsx
+++ b/apps/sociaal-wonen/public/data/sociaal-wonen-alle-gegevens.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gegevens" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toelichting" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gegevens" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Toelichting" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26621,7 +26621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -26704,132 +26704,118 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Interne dossiernummers (Woonproject, Verrichting) staan niet in dit bestand. De SSI-bladen zijn niet inbegrepen, omdat ze overlappen met de gewone planning.</t>
-        </is>
-      </c>
+      <c r="A13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr"/>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Kolommen</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Kolommen</t>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Huurwoningen: Aantal huurwoningen dat zal gerealiseerd worden. Bij renovatie gaat het om bestaande woningen waarvan de ingreep beperkt kan zijn (bv. raamcontracten of beperkte renovatie). Vergelijk bedragen per woning daarom enkel binnen hetzelfde soort werken.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Huurwoningen: Aantal huurwoningen dat zal gerealiseerd worden. Bij renovatie gaat het om bestaande woningen waarvan de ingreep beperkt kan zijn (bv. raamcontracten of beperkte renovatie). Vergelijk bedragen per woning daarom enkel binnen hetzelfde soort werken.</t>
+          <t>Kostprijs (EUR): Geraamde kostprijs van de werken.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Kostprijs (EUR): Geraamde kostprijs van de werken.</t>
+          <t>Maximumprijs VMSW (EUR): FS4-plafond. Niet voor elke rij ingevuld.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Maximumprijs VMSW (EUR): FS4-plafond. Niet voor elke rij ingevuld.</t>
+          <t>Bedrag UP (EUR): Subsidiabel bedrag (berekend op basis van kostprijs en maximumprijs).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Bedrag UP (EUR): Subsidiabel bedrag (berekend op basis van kostprijs en maximumprijs).</t>
+          <t>Datum opname programmatie: Datum opname programmatie (kolom Datum Beslissing in de bron).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Datum opname programmatie: Datum opname programmatie (kolom Datum Beslissing in de bron).</t>
+          <t>Procedure: de kolom Extra info uit de bron, bv. CBO, Modulair Wonen, Design &amp; Build, raamcontract, beperkte renovatie. Leeg als niets vermeld is.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Procedure: de kolom Extra info uit de bron, bv. CBO, Modulair Wonen, Design &amp; Build, raamcontract, beperkte renovatie. Leeg als niets vermeld is.</t>
+          <t>Aantal verrichtingen: aantal verrichtingen achter de rij (1 bij niveau Project).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Aantal verrichtingen: aantal verrichtingen achter de rij (1 bij niveau Project).</t>
+          <t>Provincie en gemeente zijn afgeleid uit de NIS-code van de gemeente, niet uit de bronkolom. Rijen zonder eenduidige gemeente hebben geen NIS-code.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Provincie en gemeente zijn afgeleid uit de NIS-code van de gemeente, niet uit de bronkolom. Rijen zonder eenduidige gemeente hebben geen NIS-code.</t>
-        </is>
-      </c>
+      <c r="A23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Herhaalde huurwaarden binnen een verrichting zijn niet gecorrigeerd, zodat de totalen overeenkomen met de totaalrijen van VMSW.</t>
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Types verrichting</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>NB: Nieuwbouw</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Types verrichting</t>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>VVP: Vervangingsbouw verworven patrimonium</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>NB: Nieuwbouw</t>
+          <t>RVP: Renovatie verworven patrimonium</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>VVP: Vervangingsbouw verworven patrimonium</t>
+          <t>GW: Aankoop goede woning</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>RVP: Renovatie verworven patrimonium</t>
+          <t>VEP: Vervangingsbouw eigen patrimonium</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>GW: Aankoop goede woning</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>VEP: Vervangingsbouw eigen patrimonium</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>REP: Renovatie eigen patrimonium</t>
         </is>

</xml_diff>

<commit_message>
feat(sociaal-wonen): separate limited renovations
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/apps/sociaal-wonen/public/data/sociaal-wonen-alle-gegevens.xlsx
+++ b/apps/sociaal-wonen/public/data/sociaal-wonen-alle-gegevens.xlsx
@@ -482,7 +482,7 @@
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="39" customWidth="1" min="9" max="9"/>
     <col width="33" customWidth="1" min="10" max="10"/>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3636,7 +3636,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -5882,7 +5882,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -5957,7 +5957,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -6247,7 +6247,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -6385,7 +6385,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -6610,7 +6610,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -6685,7 +6685,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -7125,7 +7125,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -7200,7 +7200,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -7915,7 +7915,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -7990,7 +7990,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -8065,7 +8065,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -8135,7 +8135,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -8205,7 +8205,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -8280,7 +8280,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -9006,7 +9006,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -9361,7 +9361,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -9644,7 +9644,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -9859,7 +9859,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -9934,7 +9934,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -10009,7 +10009,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -10574,7 +10574,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Renovatie</t>
+          <t>Beperkte renovatie</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -26621,7 +26621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -26716,106 +26716,113 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Huurwoningen: Aantal huurwoningen dat zal gerealiseerd worden. Bij renovatie gaat het om bestaande woningen waarvan de ingreep beperkt kan zijn (bv. raamcontracten of beperkte renovatie). Vergelijk bedragen per woning daarom enkel binnen hetzelfde soort werken.</t>
+          <t>Soort werken: renovaties met 'Beperkte renovatie' in de kolom Extra info worden als aparte categorie getoond. Raamcontracten blijven opgenomen; de categorie wordt niet dubbel geteld.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Kostprijs (EUR): Geraamde kostprijs van de werken.</t>
+          <t>Huurwoningen: Aantal huurwoningen dat zal gerealiseerd worden. Bij renovatie gaat het om bestaande woningen. Het aantal zegt bij beperkte renovaties en raamcontracten weinig over de omvang van de ingreep. Vergelijk bedragen per woning daarom enkel binnen hetzelfde soort werken.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Maximumprijs VMSW (EUR): FS4-plafond. Niet voor elke rij ingevuld.</t>
+          <t>Kostprijs (EUR): Geraamde kostprijs van de werken.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Bedrag UP (EUR): Subsidiabel bedrag (berekend op basis van kostprijs en maximumprijs).</t>
+          <t>Maximumprijs VMSW (EUR): FS4-plafond. Niet voor elke rij ingevuld.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Datum opname programmatie: Datum opname programmatie (kolom Datum Beslissing in de bron).</t>
+          <t>Bedrag UP (EUR): Subsidiabel bedrag (berekend op basis van kostprijs en maximumprijs).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Procedure: de kolom Extra info uit de bron, bv. CBO, Modulair Wonen, Design &amp; Build, raamcontract, beperkte renovatie. Leeg als niets vermeld is.</t>
+          <t>Datum opname programmatie: Datum opname programmatie (kolom Datum Beslissing in de bron).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Aantal verrichtingen: aantal verrichtingen achter de rij (1 bij niveau Project).</t>
+          <t>Procedure: de kolom Extra info uit de bron, bv. CBO, Modulair Wonen, Design &amp; Build, raamcontract, beperkte renovatie. Leeg als niets vermeld is.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>Aantal verrichtingen: aantal verrichtingen achter de rij (1 bij niveau Project).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>Provincie en gemeente zijn afgeleid uit de NIS-code van de gemeente, niet uit de bronkolom. Rijen zonder eenduidige gemeente hebben geen NIS-code.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Types verrichting</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>NB: Nieuwbouw</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>VVP: Vervangingsbouw verworven patrimonium</t>
+          <t>NB: Nieuwbouw</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>RVP: Renovatie verworven patrimonium</t>
+          <t>VVP: Vervangingsbouw verworven patrimonium</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>GW: Aankoop goede woning</t>
+          <t>RVP: Renovatie verworven patrimonium</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>VEP: Vervangingsbouw eigen patrimonium</t>
+          <t>GW: Aankoop goede woning</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>VEP: Vervangingsbouw eigen patrimonium</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>REP: Renovatie eigen patrimonium</t>
         </is>

</xml_diff>